<commit_message>
Sync planning SharePoint : S46
</commit_message>
<xml_diff>
--- a/Plannings 2026 S46.xlsx
+++ b/Plannings 2026 S46.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3140DCD-9426-4C32-8EE9-BB8F9EFFEED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{B3140DCD-9426-4C32-8EE9-BB8F9EFFEED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D991FA3-09C5-4183-B0ED-251389945260}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6598,7 +6598,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="38" t="s">
         <v>40</v>
       </c>
       <c r="C25" s="38" t="s">
@@ -6616,7 +6616,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="39" t="s">
         <v>44</v>
       </c>
       <c r="C26" s="39" t="s">
@@ -6634,7 +6634,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
-      <c r="B27" s="42"/>
+      <c r="B27" s="39"/>
       <c r="C27" s="38" t="s">
         <v>40</v>
       </c>
@@ -6648,7 +6648,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="25"/>
-      <c r="B28" s="42"/>
+      <c r="B28" s="39"/>
       <c r="C28" s="39" t="s">
         <v>48</v>
       </c>
@@ -6662,7 +6662,7 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="25"/>
-      <c r="B29" s="42"/>
+      <c r="B29" s="39"/>
       <c r="C29" s="41" t="s">
         <v>40</v>
       </c>
@@ -6676,7 +6676,7 @@
     </row>
     <row r="30" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="27"/>
-      <c r="B30" s="43"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="43" t="s">
         <v>50</v>
       </c>
@@ -8342,13 +8342,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A20AAC2-369B-4699-8644-4367F4F0E3A8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A670DFB3-4E88-4AF2-B690-D1C73746BF68}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40E103B2-006F-47F4-8EFF-D92C4A239073}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B70CBE5F-0055-4F1B-9CB9-7149C52E83D7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C889D4AA-2256-47B4-B8F5-7358D1D49ED3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3632A59-1026-4BBC-90EB-ED690FF88C9C}"/>
 </file>
</xml_diff>